<commit_message>
Cashflow: make design, website, photos and load test DIY
Zeroes those launch costs, keeps their old estimates in the notes, and
lowers the default founder injection to R40,000 to match the smaller
cash need.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PFa8GoAoTQbC8BRtnWoPyP
</commit_message>
<xml_diff>
--- a/Big Jos Beds 12-month cashflow.xlsx
+++ b/Big Jos Beds 12-month cashflow.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="169">
   <si>
     <t xml:space="preserve">Big Jo's Beds: 12-month bootstrap cashflow plan</t>
   </si>
@@ -335,15 +335,21 @@
     <t xml:space="preserve">Brand identity and label design</t>
   </si>
   <si>
-    <t xml:space="preserve">Estimate, freelance designer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Website build (Shopify theme and setup)</t>
+    <t xml:space="preserve">DIY. A freelance designer was estimated at R20,000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Website build</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIY on Shopify. The Shopify plan is still in fixed costs. Was R10,000</t>
   </si>
   <si>
     <t xml:space="preserve">Photo and video shoot</t>
   </si>
   <si>
+    <t xml:space="preserve">DIY. Was R8,000</t>
+  </si>
+  <si>
     <t xml:space="preserve">Branded side-panel label setup</t>
   </si>
   <si>
@@ -356,10 +362,10 @@
     <t xml:space="preserve">Launch activation (e.g. a Get Lucky golf day stand)</t>
   </si>
   <si>
-    <t xml:space="preserve">Independent 250 kg durability test</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estimate. Get an SABS or university lab quote</t>
+    <t xml:space="preserve">250 kg durability test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIY, so not independent proof. An SABS or university lab test was estimated at R25,000</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -1254,15 +1260,15 @@
       </c>
       <c r="B14" s="7" t="n">
         <f aca="false">'Slow case'!B32</f>
-        <v>-83380</v>
+        <v>-20380</v>
       </c>
       <c r="C14" s="7" t="n">
         <f aca="false">'Base case'!B32</f>
-        <v>-83380</v>
+        <v>-20380</v>
       </c>
       <c r="D14" s="7" t="n">
         <f aca="false">'Target case'!B32</f>
-        <v>-83380</v>
+        <v>-20380</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1288,15 +1294,15 @@
       </c>
       <c r="B16" s="9" t="n">
         <f aca="false">'Slow case'!B36</f>
-        <v>103122.2565</v>
+        <v>166122.2565</v>
       </c>
       <c r="C16" s="9" t="n">
         <f aca="false">'Base case'!B36</f>
-        <v>574491.6435</v>
+        <v>637491.6435</v>
       </c>
       <c r="D16" s="9" t="n">
         <f aca="false">'Target case'!B36</f>
-        <v>1435723.56795652</v>
+        <v>1498723.56795652</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1305,15 +1311,15 @@
       </c>
       <c r="B17" s="9" t="n">
         <f aca="false">MAX(0,-MIN('Slow case'!C42:N42))</f>
-        <v>90144.009</v>
+        <v>29262.0045</v>
       </c>
       <c r="C17" s="9" t="n">
         <f aca="false">MAX(0,-MIN('Base case'!C42:N42))</f>
-        <v>50112.0045</v>
+        <v>12112.0045</v>
       </c>
       <c r="D17" s="9" t="n">
         <f aca="false">MAX(0,-MIN('Target case'!C42:N42))</f>
-        <v>35844.009</v>
+        <v>11230</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1322,15 +1328,15 @@
       </c>
       <c r="B18" s="7" t="n">
         <f aca="false">MIN('Slow case'!C39:N39)</f>
-        <v>9855.991</v>
+        <v>10737.9955</v>
       </c>
       <c r="C18" s="7" t="n">
         <f aca="false">MIN('Base case'!C39:N39)</f>
-        <v>49887.9955</v>
+        <v>27887.9955</v>
       </c>
       <c r="D18" s="7" t="n">
         <f aca="false">MIN('Target case'!C39:N39)</f>
-        <v>64155.991</v>
+        <v>28770</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1339,15 +1345,15 @@
       </c>
       <c r="B19" s="9" t="n">
         <f aca="false">'Slow case'!N39</f>
-        <v>203122.2565</v>
+        <v>206122.2565</v>
       </c>
       <c r="C19" s="9" t="n">
         <f aca="false">'Base case'!N39</f>
-        <v>674491.6435</v>
+        <v>677491.6435</v>
       </c>
       <c r="D19" s="9" t="n">
         <f aca="false">'Target case'!N39</f>
-        <v>1535723.56795652</v>
+        <v>1538723.56795652</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1356,15 +1362,15 @@
       </c>
       <c r="B20" s="10" t="str">
         <f aca="false">IFERROR(INDEX('Slow case'!C5:N5,MATCH(1,'Slow case'!C45:N45,0)),"Not in 12 months")</f>
-        <v>Jul 2027</v>
+        <v>Apr 2027</v>
       </c>
       <c r="C20" s="10" t="str">
         <f aca="false">IFERROR(INDEX('Base case'!C5:N5,MATCH(1,'Base case'!C45:N45,0)),"Not in 12 months")</f>
-        <v>Mar 2027</v>
+        <v>Jan 2027</v>
       </c>
       <c r="D20" s="10" t="str">
         <f aca="false">IFERROR(INDEX('Target case'!C5:N5,MATCH(1,'Target case'!C45:N45,0)),"Not in 12 months")</f>
-        <v>Dec 2026</v>
+        <v>Nov 2026</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1472,51 +1478,51 @@
       </c>
       <c r="B27" s="14" t="n">
         <f aca="false">'Slow case'!C39</f>
-        <v>68770</v>
+        <v>28770</v>
       </c>
       <c r="C27" s="14" t="n">
         <f aca="false">'Slow case'!D39</f>
-        <v>35620</v>
+        <v>13620</v>
       </c>
       <c r="D27" s="14" t="n">
         <f aca="false">'Slow case'!E39</f>
-        <v>32737.9955</v>
+        <v>10737.9955</v>
       </c>
       <c r="E27" s="14" t="n">
         <f aca="false">'Slow case'!F39</f>
-        <v>9855.991</v>
+        <v>12855.991</v>
       </c>
       <c r="F27" s="14" t="n">
         <f aca="false">'Slow case'!G39</f>
-        <v>11973.9865</v>
+        <v>14973.9865</v>
       </c>
       <c r="G27" s="14" t="n">
         <f aca="false">'Slow case'!H39</f>
-        <v>27596.5075</v>
+        <v>30596.5075</v>
       </c>
       <c r="H27" s="14" t="n">
         <f aca="false">'Slow case'!I39</f>
-        <v>43219.0285</v>
+        <v>46219.0285</v>
       </c>
       <c r="I27" s="14" t="n">
         <f aca="false">'Slow case'!J39</f>
-        <v>58841.5495</v>
+        <v>61841.5495</v>
       </c>
       <c r="J27" s="14" t="n">
         <f aca="false">'Slow case'!K39</f>
-        <v>87968.596</v>
+        <v>90968.596</v>
       </c>
       <c r="K27" s="14" t="n">
         <f aca="false">'Slow case'!L39</f>
-        <v>117095.6425</v>
+        <v>120095.6425</v>
       </c>
       <c r="L27" s="14" t="n">
         <f aca="false">'Slow case'!M39</f>
-        <v>160490.6845</v>
+        <v>163490.6845</v>
       </c>
       <c r="M27" s="14" t="n">
         <f aca="false">'Slow case'!N39</f>
-        <v>203122.2565</v>
+        <v>206122.2565</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1525,51 +1531,51 @@
       </c>
       <c r="B28" s="14" t="n">
         <f aca="false">'Base case'!C39</f>
-        <v>68770</v>
+        <v>28770</v>
       </c>
       <c r="C28" s="14" t="n">
         <f aca="false">'Base case'!D39</f>
-        <v>49887.9955</v>
+        <v>27887.9955</v>
       </c>
       <c r="D28" s="14" t="n">
         <f aca="false">'Base case'!E39</f>
-        <v>61273.9865</v>
+        <v>39273.9865</v>
       </c>
       <c r="E28" s="14" t="n">
         <f aca="false">'Base case'!F39</f>
-        <v>52659.9775</v>
+        <v>55659.9775</v>
       </c>
       <c r="F28" s="14" t="n">
         <f aca="false">'Base case'!G39</f>
-        <v>82550.494</v>
+        <v>85550.494</v>
       </c>
       <c r="G28" s="14" t="n">
         <f aca="false">'Base case'!H39</f>
-        <v>125945.536</v>
+        <v>128945.536</v>
       </c>
       <c r="H28" s="14" t="n">
         <f aca="false">'Base case'!I39</f>
-        <v>183608.5735</v>
+        <v>186608.5735</v>
       </c>
       <c r="I28" s="14" t="n">
         <f aca="false">'Base case'!J39</f>
-        <v>254776.1365</v>
+        <v>257776.1365</v>
       </c>
       <c r="J28" s="14" t="n">
         <f aca="false">'Base case'!K39</f>
-        <v>339448.225</v>
+        <v>342448.225</v>
       </c>
       <c r="K28" s="14" t="n">
         <f aca="false">'Base case'!L39</f>
-        <v>437624.839</v>
+        <v>440624.839</v>
       </c>
       <c r="L28" s="14" t="n">
         <f aca="false">'Base case'!M39</f>
-        <v>549305.9785</v>
+        <v>552305.9785</v>
       </c>
       <c r="M28" s="14" t="n">
         <f aca="false">'Base case'!N39</f>
-        <v>674491.6435</v>
+        <v>677491.6435</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1578,51 +1584,51 @@
       </c>
       <c r="B29" s="14" t="n">
         <f aca="false">'Target case'!C39</f>
-        <v>68770</v>
+        <v>28770</v>
       </c>
       <c r="C29" s="14" t="n">
         <f aca="false">'Target case'!D39</f>
-        <v>64155.991</v>
+        <v>42155.991</v>
       </c>
       <c r="D29" s="14" t="n">
         <f aca="false">'Target case'!E39</f>
-        <v>104077.973</v>
+        <v>82077.973</v>
       </c>
       <c r="E29" s="14" t="n">
         <f aca="false">'Target case'!F39</f>
-        <v>138267.9505</v>
+        <v>141267.9505</v>
       </c>
       <c r="F29" s="14" t="n">
         <f aca="false">'Target case'!G39</f>
-        <v>224466.979</v>
+        <v>227466.979</v>
       </c>
       <c r="G29" s="14" t="n">
         <f aca="false">'Target case'!H39</f>
-        <v>337675.0585</v>
+        <v>340675.0585</v>
       </c>
       <c r="H29" s="14" t="n">
         <f aca="false">'Target case'!I39</f>
-        <v>478655.659</v>
+        <v>481655.659</v>
       </c>
       <c r="I29" s="14" t="n">
         <f aca="false">'Target case'!J39</f>
-        <v>646645.3105</v>
+        <v>649645.3105</v>
       </c>
       <c r="J29" s="14" t="n">
         <f aca="false">'Target case'!K39</f>
-        <v>841644.013</v>
+        <v>844644.013</v>
       </c>
       <c r="K29" s="14" t="n">
         <f aca="false">'Target case'!L39</f>
-        <v>1063651.7665</v>
+        <v>1066651.7665</v>
       </c>
       <c r="L29" s="14" t="n">
         <f aca="false">'Target case'!M39</f>
-        <v>1312668.571</v>
+        <v>1315668.571</v>
       </c>
       <c r="M29" s="14" t="n">
         <f aca="false">'Target case'!N39</f>
-        <v>1535723.56795652</v>
+        <v>1538723.56795652</v>
       </c>
     </row>
   </sheetData>
@@ -1979,7 +1985,7 @@
         <v>74</v>
       </c>
       <c r="B33" s="15" t="n">
-        <v>100000</v>
+        <v>40000</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>75</v>
@@ -2212,7 +2218,7 @@
         <v>102</v>
       </c>
       <c r="B52" s="16" t="n">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="C52" s="17" t="n">
         <v>1</v>
@@ -2226,32 +2232,32 @@
         <v>104</v>
       </c>
       <c r="B53" s="16" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="C53" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>39</v>
+        <v>105</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="5" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B54" s="16" t="n">
-        <v>8000</v>
+        <v>0</v>
       </c>
       <c r="C54" s="17" t="n">
         <v>2</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>39</v>
+        <v>107</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B55" s="16" t="n">
         <v>3000</v>
@@ -2260,12 +2266,12 @@
         <v>2</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B56" s="16" t="n">
         <v>2000</v>
@@ -2279,7 +2285,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="5" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B57" s="16" t="n">
         <v>5000</v>
@@ -2293,30 +2299,30 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B58" s="16" t="n">
-        <v>25000</v>
+        <v>0</v>
       </c>
       <c r="C58" s="17" t="n">
         <v>4</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="11" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B59" s="20" t="n">
         <f aca="false">SUM(B48:B58)</f>
-        <v>83380</v>
+        <v>20380</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B61" s="3"/>
       <c r="C61" s="3"/>
@@ -2337,7 +2343,7 @@
         <v>93</v>
       </c>
       <c r="B62" s="11" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C62" s="21" t="n">
         <v>1</v>
@@ -2381,45 +2387,45 @@
         <v>26</v>
       </c>
       <c r="C63" s="22" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D63" s="22" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="E63" s="22" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F63" s="22" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="G63" s="22" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="H63" s="22" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="I63" s="22" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="J63" s="22" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="K63" s="22" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="L63" s="22" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="M63" s="22" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="N63" s="22" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B64" s="23" t="n">
         <f aca="false">SUM(C64:N64)</f>
@@ -2464,12 +2470,12 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="11" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B67" s="24" t="n">
         <f aca="false">SUM(C67:N67)</f>
@@ -2514,7 +2520,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B68" s="24" t="n">
         <f aca="false">SUM(C68:N68)</f>
@@ -2559,7 +2565,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B69" s="24" t="n">
         <f aca="false">SUM(C69:N69)</f>
@@ -2604,7 +2610,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="2" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -2633,18 +2639,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B2" s="26" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2705,7 +2711,7 @@
         <v>26</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C5" s="13" t="str">
         <f aca="false">Assumptions!C63</f>
@@ -2815,7 +2821,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C7" s="14" t="n">
         <f aca="false">IF(C$4&gt;=Assumptions!$B$7,Assumptions!$B$6,Assumptions!$B$5)</f>
@@ -2868,7 +2874,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -2886,7 +2892,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B10" s="30" t="n">
         <f aca="false">SUM(C10:N10)</f>
@@ -2943,7 +2949,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B11" s="30" t="n">
         <f aca="false">SUM(C11:N11)</f>
@@ -3057,7 +3063,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B13" s="31" t="n">
         <f aca="false">SUM(C13:N13)</f>
@@ -3114,7 +3120,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -3132,7 +3138,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B16" s="30" t="n">
         <f aca="false">SUM(C16:N16)</f>
@@ -3189,7 +3195,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B17" s="30" t="n">
         <f aca="false">SUM(C17:N17)</f>
@@ -3246,7 +3252,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B18" s="30" t="n">
         <f aca="false">SUM(C18:N18)</f>
@@ -3303,7 +3309,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B19" s="30" t="n">
         <f aca="false">SUM(C19:N19)</f>
@@ -3360,7 +3366,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B20" s="30" t="n">
         <f aca="false">SUM(C20:N20)</f>
@@ -3474,7 +3480,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B22" s="30" t="n">
         <f aca="false">SUM(C22:N22)</f>
@@ -3531,7 +3537,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B23" s="30" t="n">
         <f aca="false">SUM(C23:N23)</f>
@@ -3588,7 +3594,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B24" s="30" t="n">
         <f aca="false">SUM(C24:N24)</f>
@@ -3645,7 +3651,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B25" s="31" t="n">
         <f aca="false">SUM(C25:N25)</f>
@@ -3759,7 +3765,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -3895,15 +3901,15 @@
       </c>
       <c r="B32" s="30" t="n">
         <f aca="false">SUM(C32:N32)</f>
-        <v>-83380</v>
+        <v>-20380</v>
       </c>
       <c r="C32" s="30" t="n">
         <f aca="false">-SUMIF(Assumptions!$C$48:$C$58,C$4,Assumptions!$B$48:$B$58)</f>
-        <v>-30380</v>
+        <v>-10380</v>
       </c>
       <c r="D32" s="30" t="n">
         <f aca="false">-SUMIF(Assumptions!$C$48:$C$58,D$4,Assumptions!$B$48:$B$58)</f>
-        <v>-23000</v>
+        <v>-5000</v>
       </c>
       <c r="E32" s="30" t="n">
         <f aca="false">-SUMIF(Assumptions!$C$48:$C$58,E$4,Assumptions!$B$48:$B$58)</f>
@@ -3911,7 +3917,7 @@
       </c>
       <c r="F32" s="30" t="n">
         <f aca="false">-SUMIF(Assumptions!$C$48:$C$58,F$4,Assumptions!$B$48:$B$58)</f>
-        <v>-25000</v>
+        <v>-0</v>
       </c>
       <c r="G32" s="30" t="n">
         <f aca="false">-SUMIF(Assumptions!$C$48:$C$58,G$4,Assumptions!$B$48:$B$58)</f>
@@ -3948,7 +3954,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B33" s="30" t="n">
         <f aca="false">SUM(C33:N33)</f>
@@ -4005,19 +4011,19 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="8" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B34" s="31" t="n">
         <f aca="false">SUM(C34:N34)</f>
-        <v>-215880</v>
+        <v>-152880</v>
       </c>
       <c r="C34" s="31" t="n">
         <f aca="false">SUM(C30:C33)</f>
-        <v>-31230</v>
+        <v>-11230</v>
       </c>
       <c r="D34" s="31" t="n">
         <f aca="false">SUM(D30:D33)</f>
-        <v>-33150</v>
+        <v>-15150</v>
       </c>
       <c r="E34" s="31" t="n">
         <f aca="false">SUM(E30:E33)</f>
@@ -4025,7 +4031,7 @@
       </c>
       <c r="F34" s="31" t="n">
         <f aca="false">SUM(F30:F33)</f>
-        <v>-37150</v>
+        <v>-12150</v>
       </c>
       <c r="G34" s="31" t="n">
         <f aca="false">SUM(G30:G33)</f>
@@ -4062,19 +4068,19 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="8" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B36" s="31" t="n">
         <f aca="false">SUM(C36:N36)</f>
-        <v>103122.2565</v>
+        <v>166122.2565</v>
       </c>
       <c r="C36" s="31" t="n">
         <f aca="false">C27+C34</f>
-        <v>-31230</v>
+        <v>-11230</v>
       </c>
       <c r="D36" s="31" t="n">
         <f aca="false">D27+D34</f>
-        <v>-33150</v>
+        <v>-15150</v>
       </c>
       <c r="E36" s="31" t="n">
         <f aca="false">E27+E34</f>
@@ -4082,7 +4088,7 @@
       </c>
       <c r="F36" s="31" t="n">
         <f aca="false">F27+F34</f>
-        <v>-22882.0045</v>
+        <v>2117.9955</v>
       </c>
       <c r="G36" s="31" t="n">
         <f aca="false">G27+G34</f>
@@ -4123,11 +4129,11 @@
       </c>
       <c r="B37" s="30" t="n">
         <f aca="false">SUM(C37:N37)</f>
-        <v>100000</v>
+        <v>40000</v>
       </c>
       <c r="C37" s="30" t="n">
         <f aca="false">IF(C$4=Assumptions!$B$34,Assumptions!$B$33,0)</f>
-        <v>100000</v>
+        <v>40000</v>
       </c>
       <c r="D37" s="30" t="n">
         <f aca="false">IF(D$4=Assumptions!$B$34,Assumptions!$B$33,0)</f>
@@ -4176,7 +4182,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C38" s="30" t="n">
         <f aca="false">0</f>
@@ -4184,106 +4190,106 @@
       </c>
       <c r="D38" s="30" t="n">
         <f aca="false">C39</f>
-        <v>68770</v>
+        <v>28770</v>
       </c>
       <c r="E38" s="30" t="n">
         <f aca="false">D39</f>
-        <v>35620</v>
+        <v>13620</v>
       </c>
       <c r="F38" s="30" t="n">
         <f aca="false">E39</f>
-        <v>32737.9955</v>
+        <v>10737.9955</v>
       </c>
       <c r="G38" s="30" t="n">
         <f aca="false">F39</f>
-        <v>9855.991</v>
+        <v>12855.991</v>
       </c>
       <c r="H38" s="30" t="n">
         <f aca="false">G39</f>
-        <v>11973.9865</v>
+        <v>14973.9865</v>
       </c>
       <c r="I38" s="30" t="n">
         <f aca="false">H39</f>
-        <v>27596.5075</v>
+        <v>30596.5075</v>
       </c>
       <c r="J38" s="30" t="n">
         <f aca="false">I39</f>
-        <v>43219.0285</v>
+        <v>46219.0285</v>
       </c>
       <c r="K38" s="30" t="n">
         <f aca="false">J39</f>
-        <v>58841.5495</v>
+        <v>61841.5495</v>
       </c>
       <c r="L38" s="30" t="n">
         <f aca="false">K39</f>
-        <v>87968.596</v>
+        <v>90968.596</v>
       </c>
       <c r="M38" s="30" t="n">
         <f aca="false">L39</f>
-        <v>117095.6425</v>
+        <v>120095.6425</v>
       </c>
       <c r="N38" s="30" t="n">
         <f aca="false">M39</f>
-        <v>160490.6845</v>
+        <v>163490.6845</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="8" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B39" s="32"/>
       <c r="C39" s="31" t="n">
         <f aca="false">C38+C36+C37</f>
-        <v>68770</v>
+        <v>28770</v>
       </c>
       <c r="D39" s="31" t="n">
         <f aca="false">D38+D36+D37</f>
-        <v>35620</v>
+        <v>13620</v>
       </c>
       <c r="E39" s="31" t="n">
         <f aca="false">E38+E36+E37</f>
-        <v>32737.9955</v>
+        <v>10737.9955</v>
       </c>
       <c r="F39" s="31" t="n">
         <f aca="false">F38+F36+F37</f>
-        <v>9855.991</v>
+        <v>12855.991</v>
       </c>
       <c r="G39" s="31" t="n">
         <f aca="false">G38+G36+G37</f>
-        <v>11973.9865</v>
+        <v>14973.9865</v>
       </c>
       <c r="H39" s="31" t="n">
         <f aca="false">H38+H36+H37</f>
-        <v>27596.5075</v>
+        <v>30596.5075</v>
       </c>
       <c r="I39" s="31" t="n">
         <f aca="false">I38+I36+I37</f>
-        <v>43219.0285</v>
+        <v>46219.0285</v>
       </c>
       <c r="J39" s="31" t="n">
         <f aca="false">J38+J36+J37</f>
-        <v>58841.5495</v>
+        <v>61841.5495</v>
       </c>
       <c r="K39" s="31" t="n">
         <f aca="false">K38+K36+K37</f>
-        <v>87968.596</v>
+        <v>90968.596</v>
       </c>
       <c r="L39" s="31" t="n">
         <f aca="false">L38+L36+L37</f>
-        <v>117095.6425</v>
+        <v>120095.6425</v>
       </c>
       <c r="M39" s="31" t="n">
         <f aca="false">M38+M36+M37</f>
-        <v>160490.6845</v>
+        <v>163490.6845</v>
       </c>
       <c r="N39" s="31" t="n">
         <f aca="false">N38+N36+N37</f>
-        <v>203122.2565</v>
+        <v>206122.2565</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
@@ -4301,60 +4307,60 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C42" s="30" t="n">
         <f aca="false">C36</f>
-        <v>-31230</v>
+        <v>-11230</v>
       </c>
       <c r="D42" s="30" t="n">
         <f aca="false">C42+D36</f>
-        <v>-64380</v>
+        <v>-26380</v>
       </c>
       <c r="E42" s="30" t="n">
         <f aca="false">D42+E36</f>
-        <v>-67262.0045</v>
+        <v>-29262.0045</v>
       </c>
       <c r="F42" s="30" t="n">
         <f aca="false">E42+F36</f>
-        <v>-90144.009</v>
+        <v>-27144.009</v>
       </c>
       <c r="G42" s="30" t="n">
         <f aca="false">F42+G36</f>
-        <v>-88026.0135</v>
+        <v>-25026.0135</v>
       </c>
       <c r="H42" s="30" t="n">
         <f aca="false">G42+H36</f>
-        <v>-72403.4925</v>
+        <v>-9403.4925</v>
       </c>
       <c r="I42" s="30" t="n">
         <f aca="false">H42+I36</f>
-        <v>-56780.9715</v>
+        <v>6219.0285</v>
       </c>
       <c r="J42" s="30" t="n">
         <f aca="false">I42+J36</f>
-        <v>-41158.4505</v>
+        <v>21841.5495</v>
       </c>
       <c r="K42" s="30" t="n">
         <f aca="false">J42+K36</f>
-        <v>-12031.404</v>
+        <v>50968.596</v>
       </c>
       <c r="L42" s="30" t="n">
         <f aca="false">K42+L36</f>
-        <v>17095.6425</v>
+        <v>80095.6425</v>
       </c>
       <c r="M42" s="30" t="n">
         <f aca="false">L42+M36</f>
-        <v>60490.6845</v>
+        <v>123490.6845</v>
       </c>
       <c r="N42" s="30" t="n">
         <f aca="false">M42+N36</f>
-        <v>103122.2565</v>
+        <v>166122.2565</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C43" s="30" t="n">
         <f aca="false">C10+C11</f>
@@ -4407,7 +4413,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C44" s="33" t="n">
         <f aca="false">IF(C43&gt;Assumptions!$B$29,1,0)</f>
@@ -4460,7 +4466,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C45" s="33" t="n">
         <f aca="false">IF(C42&gt;=0,1,0)</f>
@@ -4488,15 +4494,15 @@
       </c>
       <c r="I45" s="33" t="n">
         <f aca="false">IF(I42&gt;=0,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J45" s="33" t="n">
         <f aca="false">IF(J42&gt;=0,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K45" s="33" t="n">
         <f aca="false">IF(K42&gt;=0,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L45" s="33" t="n">
         <f aca="false">IF(L42&gt;=0,1,0)</f>
@@ -4513,19 +4519,19 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B46" s="34" t="n">
         <f aca="false">MIN(Assumptions!B30,IFERROR(MATCH(1,C44:N44,0)+1,13))</f>
         <v>13</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
   </sheetData>
@@ -4554,18 +4560,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B2" s="26" t="n">
         <v>2</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4626,7 +4632,7 @@
         <v>26</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C5" s="13" t="str">
         <f aca="false">Assumptions!C63</f>
@@ -4736,7 +4742,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C7" s="14" t="n">
         <f aca="false">IF(C$4&gt;=Assumptions!$B$7,Assumptions!$B$6,Assumptions!$B$5)</f>
@@ -4789,7 +4795,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -4807,7 +4813,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B10" s="30" t="n">
         <f aca="false">SUM(C10:N10)</f>
@@ -4864,7 +4870,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B11" s="30" t="n">
         <f aca="false">SUM(C11:N11)</f>
@@ -4978,7 +4984,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B13" s="31" t="n">
         <f aca="false">SUM(C13:N13)</f>
@@ -5035,7 +5041,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -5053,7 +5059,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B16" s="30" t="n">
         <f aca="false">SUM(C16:N16)</f>
@@ -5110,7 +5116,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B17" s="30" t="n">
         <f aca="false">SUM(C17:N17)</f>
@@ -5167,7 +5173,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B18" s="30" t="n">
         <f aca="false">SUM(C18:N18)</f>
@@ -5224,7 +5230,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B19" s="30" t="n">
         <f aca="false">SUM(C19:N19)</f>
@@ -5281,7 +5287,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B20" s="30" t="n">
         <f aca="false">SUM(C20:N20)</f>
@@ -5395,7 +5401,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B22" s="30" t="n">
         <f aca="false">SUM(C22:N22)</f>
@@ -5452,7 +5458,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B23" s="30" t="n">
         <f aca="false">SUM(C23:N23)</f>
@@ -5509,7 +5515,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B24" s="30" t="n">
         <f aca="false">SUM(C24:N24)</f>
@@ -5566,7 +5572,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B25" s="31" t="n">
         <f aca="false">SUM(C25:N25)</f>
@@ -5680,7 +5686,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -5816,15 +5822,15 @@
       </c>
       <c r="B32" s="30" t="n">
         <f aca="false">SUM(C32:N32)</f>
-        <v>-83380</v>
+        <v>-20380</v>
       </c>
       <c r="C32" s="30" t="n">
         <f aca="false">-SUMIF(Assumptions!$C$48:$C$58,C$4,Assumptions!$B$48:$B$58)</f>
-        <v>-30380</v>
+        <v>-10380</v>
       </c>
       <c r="D32" s="30" t="n">
         <f aca="false">-SUMIF(Assumptions!$C$48:$C$58,D$4,Assumptions!$B$48:$B$58)</f>
-        <v>-23000</v>
+        <v>-5000</v>
       </c>
       <c r="E32" s="30" t="n">
         <f aca="false">-SUMIF(Assumptions!$C$48:$C$58,E$4,Assumptions!$B$48:$B$58)</f>
@@ -5832,7 +5838,7 @@
       </c>
       <c r="F32" s="30" t="n">
         <f aca="false">-SUMIF(Assumptions!$C$48:$C$58,F$4,Assumptions!$B$48:$B$58)</f>
-        <v>-25000</v>
+        <v>-0</v>
       </c>
       <c r="G32" s="30" t="n">
         <f aca="false">-SUMIF(Assumptions!$C$48:$C$58,G$4,Assumptions!$B$48:$B$58)</f>
@@ -5869,7 +5875,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B33" s="30" t="n">
         <f aca="false">SUM(C33:N33)</f>
@@ -5926,19 +5932,19 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="8" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B34" s="31" t="n">
         <f aca="false">SUM(C34:N34)</f>
-        <v>-215880</v>
+        <v>-152880</v>
       </c>
       <c r="C34" s="31" t="n">
         <f aca="false">SUM(C30:C33)</f>
-        <v>-31230</v>
+        <v>-11230</v>
       </c>
       <c r="D34" s="31" t="n">
         <f aca="false">SUM(D30:D33)</f>
-        <v>-33150</v>
+        <v>-15150</v>
       </c>
       <c r="E34" s="31" t="n">
         <f aca="false">SUM(E30:E33)</f>
@@ -5946,7 +5952,7 @@
       </c>
       <c r="F34" s="31" t="n">
         <f aca="false">SUM(F30:F33)</f>
-        <v>-37150</v>
+        <v>-12150</v>
       </c>
       <c r="G34" s="31" t="n">
         <f aca="false">SUM(G30:G33)</f>
@@ -5983,19 +5989,19 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="8" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B36" s="31" t="n">
         <f aca="false">SUM(C36:N36)</f>
-        <v>574491.6435</v>
+        <v>637491.6435</v>
       </c>
       <c r="C36" s="31" t="n">
         <f aca="false">C27+C34</f>
-        <v>-31230</v>
+        <v>-11230</v>
       </c>
       <c r="D36" s="31" t="n">
         <f aca="false">D27+D34</f>
-        <v>-18882.0045</v>
+        <v>-882.004499999999</v>
       </c>
       <c r="E36" s="31" t="n">
         <f aca="false">E27+E34</f>
@@ -6003,7 +6009,7 @@
       </c>
       <c r="F36" s="31" t="n">
         <f aca="false">F27+F34</f>
-        <v>-8614.009</v>
+        <v>16385.991</v>
       </c>
       <c r="G36" s="31" t="n">
         <f aca="false">G27+G34</f>
@@ -6044,11 +6050,11 @@
       </c>
       <c r="B37" s="30" t="n">
         <f aca="false">SUM(C37:N37)</f>
-        <v>100000</v>
+        <v>40000</v>
       </c>
       <c r="C37" s="30" t="n">
         <f aca="false">IF(C$4=Assumptions!$B$34,Assumptions!$B$33,0)</f>
-        <v>100000</v>
+        <v>40000</v>
       </c>
       <c r="D37" s="30" t="n">
         <f aca="false">IF(D$4=Assumptions!$B$34,Assumptions!$B$33,0)</f>
@@ -6097,7 +6103,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C38" s="30" t="n">
         <f aca="false">0</f>
@@ -6105,106 +6111,106 @@
       </c>
       <c r="D38" s="30" t="n">
         <f aca="false">C39</f>
-        <v>68770</v>
+        <v>28770</v>
       </c>
       <c r="E38" s="30" t="n">
         <f aca="false">D39</f>
-        <v>49887.9955</v>
+        <v>27887.9955</v>
       </c>
       <c r="F38" s="30" t="n">
         <f aca="false">E39</f>
-        <v>61273.9865</v>
+        <v>39273.9865</v>
       </c>
       <c r="G38" s="30" t="n">
         <f aca="false">F39</f>
-        <v>52659.9775</v>
+        <v>55659.9775</v>
       </c>
       <c r="H38" s="30" t="n">
         <f aca="false">G39</f>
-        <v>82550.494</v>
+        <v>85550.494</v>
       </c>
       <c r="I38" s="30" t="n">
         <f aca="false">H39</f>
-        <v>125945.536</v>
+        <v>128945.536</v>
       </c>
       <c r="J38" s="30" t="n">
         <f aca="false">I39</f>
-        <v>183608.5735</v>
+        <v>186608.5735</v>
       </c>
       <c r="K38" s="30" t="n">
         <f aca="false">J39</f>
-        <v>254776.1365</v>
+        <v>257776.1365</v>
       </c>
       <c r="L38" s="30" t="n">
         <f aca="false">K39</f>
-        <v>339448.225</v>
+        <v>342448.225</v>
       </c>
       <c r="M38" s="30" t="n">
         <f aca="false">L39</f>
-        <v>437624.839</v>
+        <v>440624.839</v>
       </c>
       <c r="N38" s="30" t="n">
         <f aca="false">M39</f>
-        <v>549305.9785</v>
+        <v>552305.9785</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="8" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B39" s="32"/>
       <c r="C39" s="31" t="n">
         <f aca="false">C38+C36+C37</f>
-        <v>68770</v>
+        <v>28770</v>
       </c>
       <c r="D39" s="31" t="n">
         <f aca="false">D38+D36+D37</f>
-        <v>49887.9955</v>
+        <v>27887.9955</v>
       </c>
       <c r="E39" s="31" t="n">
         <f aca="false">E38+E36+E37</f>
-        <v>61273.9865</v>
+        <v>39273.9865</v>
       </c>
       <c r="F39" s="31" t="n">
         <f aca="false">F38+F36+F37</f>
-        <v>52659.9775</v>
+        <v>55659.9775</v>
       </c>
       <c r="G39" s="31" t="n">
         <f aca="false">G38+G36+G37</f>
-        <v>82550.494</v>
+        <v>85550.494</v>
       </c>
       <c r="H39" s="31" t="n">
         <f aca="false">H38+H36+H37</f>
-        <v>125945.536</v>
+        <v>128945.536</v>
       </c>
       <c r="I39" s="31" t="n">
         <f aca="false">I38+I36+I37</f>
-        <v>183608.5735</v>
+        <v>186608.5735</v>
       </c>
       <c r="J39" s="31" t="n">
         <f aca="false">J38+J36+J37</f>
-        <v>254776.1365</v>
+        <v>257776.1365</v>
       </c>
       <c r="K39" s="31" t="n">
         <f aca="false">K38+K36+K37</f>
-        <v>339448.225</v>
+        <v>342448.225</v>
       </c>
       <c r="L39" s="31" t="n">
         <f aca="false">L38+L36+L37</f>
-        <v>437624.839</v>
+        <v>440624.839</v>
       </c>
       <c r="M39" s="31" t="n">
         <f aca="false">M38+M36+M37</f>
-        <v>549305.9785</v>
+        <v>552305.9785</v>
       </c>
       <c r="N39" s="31" t="n">
         <f aca="false">N38+N36+N37</f>
-        <v>674491.6435</v>
+        <v>677491.6435</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
@@ -6222,60 +6228,60 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C42" s="30" t="n">
         <f aca="false">C36</f>
-        <v>-31230</v>
+        <v>-11230</v>
       </c>
       <c r="D42" s="30" t="n">
         <f aca="false">C42+D36</f>
-        <v>-50112.0045</v>
+        <v>-12112.0045</v>
       </c>
       <c r="E42" s="30" t="n">
         <f aca="false">D42+E36</f>
-        <v>-38726.0135</v>
+        <v>-726.013499999997</v>
       </c>
       <c r="F42" s="30" t="n">
         <f aca="false">E42+F36</f>
-        <v>-47340.0225</v>
+        <v>15659.9775</v>
       </c>
       <c r="G42" s="30" t="n">
         <f aca="false">F42+G36</f>
-        <v>-17449.506</v>
+        <v>45550.494</v>
       </c>
       <c r="H42" s="30" t="n">
         <f aca="false">G42+H36</f>
-        <v>25945.536</v>
+        <v>88945.536</v>
       </c>
       <c r="I42" s="30" t="n">
         <f aca="false">H42+I36</f>
-        <v>83608.5735</v>
+        <v>146608.5735</v>
       </c>
       <c r="J42" s="30" t="n">
         <f aca="false">I42+J36</f>
-        <v>154776.1365</v>
+        <v>217776.1365</v>
       </c>
       <c r="K42" s="30" t="n">
         <f aca="false">J42+K36</f>
-        <v>239448.225</v>
+        <v>302448.225</v>
       </c>
       <c r="L42" s="30" t="n">
         <f aca="false">K42+L36</f>
-        <v>337624.839</v>
+        <v>400624.839</v>
       </c>
       <c r="M42" s="30" t="n">
         <f aca="false">L42+M36</f>
-        <v>449305.9785</v>
+        <v>512305.9785</v>
       </c>
       <c r="N42" s="30" t="n">
         <f aca="false">M42+N36</f>
-        <v>574491.6435</v>
+        <v>637491.6435</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C43" s="30" t="n">
         <f aca="false">C10+C11</f>
@@ -6328,7 +6334,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C44" s="33" t="n">
         <f aca="false">IF(C43&gt;Assumptions!$B$29,1,0)</f>
@@ -6381,7 +6387,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C45" s="33" t="n">
         <f aca="false">IF(C42&gt;=0,1,0)</f>
@@ -6397,11 +6403,11 @@
       </c>
       <c r="F45" s="33" t="n">
         <f aca="false">IF(F42&gt;=0,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G45" s="33" t="n">
         <f aca="false">IF(G42&gt;=0,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H45" s="33" t="n">
         <f aca="false">IF(H42&gt;=0,1,0)</f>
@@ -6434,19 +6440,19 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B46" s="34" t="n">
         <f aca="false">MIN(Assumptions!B30,IFERROR(MATCH(1,C44:N44,0)+1,13))</f>
         <v>13</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
   </sheetData>
@@ -6475,18 +6481,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B2" s="26" t="n">
         <v>3</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6547,7 +6553,7 @@
         <v>26</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C5" s="13" t="str">
         <f aca="false">Assumptions!C63</f>
@@ -6657,7 +6663,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C7" s="14" t="n">
         <f aca="false">IF(C$4&gt;=Assumptions!$B$7,Assumptions!$B$6,Assumptions!$B$5)</f>
@@ -6710,7 +6716,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -6728,7 +6734,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B10" s="30" t="n">
         <f aca="false">SUM(C10:N10)</f>
@@ -6785,7 +6791,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B11" s="30" t="n">
         <f aca="false">SUM(C11:N11)</f>
@@ -6899,7 +6905,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B13" s="31" t="n">
         <f aca="false">SUM(C13:N13)</f>
@@ -6956,7 +6962,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -6974,7 +6980,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B16" s="30" t="n">
         <f aca="false">SUM(C16:N16)</f>
@@ -7031,7 +7037,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B17" s="30" t="n">
         <f aca="false">SUM(C17:N17)</f>
@@ -7088,7 +7094,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B18" s="30" t="n">
         <f aca="false">SUM(C18:N18)</f>
@@ -7145,7 +7151,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B19" s="30" t="n">
         <f aca="false">SUM(C19:N19)</f>
@@ -7202,7 +7208,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B20" s="30" t="n">
         <f aca="false">SUM(C20:N20)</f>
@@ -7316,7 +7322,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B22" s="30" t="n">
         <f aca="false">SUM(C22:N22)</f>
@@ -7373,7 +7379,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B23" s="30" t="n">
         <f aca="false">SUM(C23:N23)</f>
@@ -7430,7 +7436,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B24" s="30" t="n">
         <f aca="false">SUM(C24:N24)</f>
@@ -7487,7 +7493,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B25" s="31" t="n">
         <f aca="false">SUM(C25:N25)</f>
@@ -7601,7 +7607,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -7737,15 +7743,15 @@
       </c>
       <c r="B32" s="30" t="n">
         <f aca="false">SUM(C32:N32)</f>
-        <v>-83380</v>
+        <v>-20380</v>
       </c>
       <c r="C32" s="30" t="n">
         <f aca="false">-SUMIF(Assumptions!$C$48:$C$58,C$4,Assumptions!$B$48:$B$58)</f>
-        <v>-30380</v>
+        <v>-10380</v>
       </c>
       <c r="D32" s="30" t="n">
         <f aca="false">-SUMIF(Assumptions!$C$48:$C$58,D$4,Assumptions!$B$48:$B$58)</f>
-        <v>-23000</v>
+        <v>-5000</v>
       </c>
       <c r="E32" s="30" t="n">
         <f aca="false">-SUMIF(Assumptions!$C$48:$C$58,E$4,Assumptions!$B$48:$B$58)</f>
@@ -7753,7 +7759,7 @@
       </c>
       <c r="F32" s="30" t="n">
         <f aca="false">-SUMIF(Assumptions!$C$48:$C$58,F$4,Assumptions!$B$48:$B$58)</f>
-        <v>-25000</v>
+        <v>-0</v>
       </c>
       <c r="G32" s="30" t="n">
         <f aca="false">-SUMIF(Assumptions!$C$48:$C$58,G$4,Assumptions!$B$48:$B$58)</f>
@@ -7790,7 +7796,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B33" s="30" t="n">
         <f aca="false">SUM(C33:N33)</f>
@@ -7847,19 +7853,19 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="8" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B34" s="31" t="n">
         <f aca="false">SUM(C34:N34)</f>
-        <v>-254582.863043478</v>
+        <v>-191582.863043478</v>
       </c>
       <c r="C34" s="31" t="n">
         <f aca="false">SUM(C30:C33)</f>
-        <v>-31230</v>
+        <v>-11230</v>
       </c>
       <c r="D34" s="31" t="n">
         <f aca="false">SUM(D30:D33)</f>
-        <v>-33150</v>
+        <v>-15150</v>
       </c>
       <c r="E34" s="31" t="n">
         <f aca="false">SUM(E30:E33)</f>
@@ -7867,7 +7873,7 @@
       </c>
       <c r="F34" s="31" t="n">
         <f aca="false">SUM(F30:F33)</f>
-        <v>-37150</v>
+        <v>-12150</v>
       </c>
       <c r="G34" s="31" t="n">
         <f aca="false">SUM(G30:G33)</f>
@@ -7904,19 +7910,19 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="8" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B36" s="31" t="n">
         <f aca="false">SUM(C36:N36)</f>
-        <v>1435723.56795652</v>
+        <v>1498723.56795652</v>
       </c>
       <c r="C36" s="31" t="n">
         <f aca="false">C27+C34</f>
-        <v>-31230</v>
+        <v>-11230</v>
       </c>
       <c r="D36" s="31" t="n">
         <f aca="false">D27+D34</f>
-        <v>-4614.009</v>
+        <v>13385.991</v>
       </c>
       <c r="E36" s="31" t="n">
         <f aca="false">E27+E34</f>
@@ -7924,7 +7930,7 @@
       </c>
       <c r="F36" s="31" t="n">
         <f aca="false">F27+F34</f>
-        <v>34189.9775</v>
+        <v>59189.9775</v>
       </c>
       <c r="G36" s="31" t="n">
         <f aca="false">G27+G34</f>
@@ -7965,11 +7971,11 @@
       </c>
       <c r="B37" s="30" t="n">
         <f aca="false">SUM(C37:N37)</f>
-        <v>100000</v>
+        <v>40000</v>
       </c>
       <c r="C37" s="30" t="n">
         <f aca="false">IF(C$4=Assumptions!$B$34,Assumptions!$B$33,0)</f>
-        <v>100000</v>
+        <v>40000</v>
       </c>
       <c r="D37" s="30" t="n">
         <f aca="false">IF(D$4=Assumptions!$B$34,Assumptions!$B$33,0)</f>
@@ -8018,7 +8024,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C38" s="30" t="n">
         <f aca="false">0</f>
@@ -8026,106 +8032,106 @@
       </c>
       <c r="D38" s="30" t="n">
         <f aca="false">C39</f>
-        <v>68770</v>
+        <v>28770</v>
       </c>
       <c r="E38" s="30" t="n">
         <f aca="false">D39</f>
-        <v>64155.991</v>
+        <v>42155.991</v>
       </c>
       <c r="F38" s="30" t="n">
         <f aca="false">E39</f>
-        <v>104077.973</v>
+        <v>82077.973</v>
       </c>
       <c r="G38" s="30" t="n">
         <f aca="false">F39</f>
-        <v>138267.9505</v>
+        <v>141267.9505</v>
       </c>
       <c r="H38" s="30" t="n">
         <f aca="false">G39</f>
-        <v>224466.979</v>
+        <v>227466.979</v>
       </c>
       <c r="I38" s="30" t="n">
         <f aca="false">H39</f>
-        <v>337675.0585</v>
+        <v>340675.0585</v>
       </c>
       <c r="J38" s="30" t="n">
         <f aca="false">I39</f>
-        <v>478655.659</v>
+        <v>481655.659</v>
       </c>
       <c r="K38" s="30" t="n">
         <f aca="false">J39</f>
-        <v>646645.3105</v>
+        <v>649645.3105</v>
       </c>
       <c r="L38" s="30" t="n">
         <f aca="false">K39</f>
-        <v>841644.013</v>
+        <v>844644.013</v>
       </c>
       <c r="M38" s="30" t="n">
         <f aca="false">L39</f>
-        <v>1063651.7665</v>
+        <v>1066651.7665</v>
       </c>
       <c r="N38" s="30" t="n">
         <f aca="false">M39</f>
-        <v>1312668.571</v>
+        <v>1315668.571</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="8" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B39" s="32"/>
       <c r="C39" s="31" t="n">
         <f aca="false">C38+C36+C37</f>
-        <v>68770</v>
+        <v>28770</v>
       </c>
       <c r="D39" s="31" t="n">
         <f aca="false">D38+D36+D37</f>
-        <v>64155.991</v>
+        <v>42155.991</v>
       </c>
       <c r="E39" s="31" t="n">
         <f aca="false">E38+E36+E37</f>
-        <v>104077.973</v>
+        <v>82077.973</v>
       </c>
       <c r="F39" s="31" t="n">
         <f aca="false">F38+F36+F37</f>
-        <v>138267.9505</v>
+        <v>141267.9505</v>
       </c>
       <c r="G39" s="31" t="n">
         <f aca="false">G38+G36+G37</f>
-        <v>224466.979</v>
+        <v>227466.979</v>
       </c>
       <c r="H39" s="31" t="n">
         <f aca="false">H38+H36+H37</f>
-        <v>337675.0585</v>
+        <v>340675.0585</v>
       </c>
       <c r="I39" s="31" t="n">
         <f aca="false">I38+I36+I37</f>
-        <v>478655.659</v>
+        <v>481655.659</v>
       </c>
       <c r="J39" s="31" t="n">
         <f aca="false">J38+J36+J37</f>
-        <v>646645.3105</v>
+        <v>649645.3105</v>
       </c>
       <c r="K39" s="31" t="n">
         <f aca="false">K38+K36+K37</f>
-        <v>841644.013</v>
+        <v>844644.013</v>
       </c>
       <c r="L39" s="31" t="n">
         <f aca="false">L38+L36+L37</f>
-        <v>1063651.7665</v>
+        <v>1066651.7665</v>
       </c>
       <c r="M39" s="31" t="n">
         <f aca="false">M38+M36+M37</f>
-        <v>1312668.571</v>
+        <v>1315668.571</v>
       </c>
       <c r="N39" s="31" t="n">
         <f aca="false">N38+N36+N37</f>
-        <v>1535723.56795652</v>
+        <v>1538723.56795652</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
@@ -8143,60 +8149,60 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C42" s="30" t="n">
         <f aca="false">C36</f>
-        <v>-31230</v>
+        <v>-11230</v>
       </c>
       <c r="D42" s="30" t="n">
         <f aca="false">C42+D36</f>
-        <v>-35844.009</v>
+        <v>2155.991</v>
       </c>
       <c r="E42" s="30" t="n">
         <f aca="false">D42+E36</f>
-        <v>4077.97300000001</v>
+        <v>42077.973</v>
       </c>
       <c r="F42" s="30" t="n">
         <f aca="false">E42+F36</f>
-        <v>38267.9505</v>
+        <v>101267.9505</v>
       </c>
       <c r="G42" s="30" t="n">
         <f aca="false">F42+G36</f>
-        <v>124466.979</v>
+        <v>187466.979</v>
       </c>
       <c r="H42" s="30" t="n">
         <f aca="false">G42+H36</f>
-        <v>237675.0585</v>
+        <v>300675.0585</v>
       </c>
       <c r="I42" s="30" t="n">
         <f aca="false">H42+I36</f>
-        <v>378655.659</v>
+        <v>441655.659</v>
       </c>
       <c r="J42" s="30" t="n">
         <f aca="false">I42+J36</f>
-        <v>546645.3105</v>
+        <v>609645.3105</v>
       </c>
       <c r="K42" s="30" t="n">
         <f aca="false">J42+K36</f>
-        <v>741644.013</v>
+        <v>804644.013</v>
       </c>
       <c r="L42" s="30" t="n">
         <f aca="false">K42+L36</f>
-        <v>963651.7665</v>
+        <v>1026651.7665</v>
       </c>
       <c r="M42" s="30" t="n">
         <f aca="false">L42+M36</f>
-        <v>1212668.571</v>
+        <v>1275668.571</v>
       </c>
       <c r="N42" s="30" t="n">
         <f aca="false">M42+N36</f>
-        <v>1435723.56795652</v>
+        <v>1498723.56795652</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C43" s="30" t="n">
         <f aca="false">C10+C11</f>
@@ -8249,7 +8255,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C44" s="33" t="n">
         <f aca="false">IF(C43&gt;Assumptions!$B$29,1,0)</f>
@@ -8302,7 +8308,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C45" s="33" t="n">
         <f aca="false">IF(C42&gt;=0,1,0)</f>
@@ -8310,7 +8316,7 @@
       </c>
       <c r="D45" s="33" t="n">
         <f aca="false">IF(D42&gt;=0,1,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E45" s="33" t="n">
         <f aca="false">IF(E42&gt;=0,1,0)</f>
@@ -8355,19 +8361,19 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B46" s="34" t="n">
         <f aca="false">MIN(Assumptions!B30,IFERROR(MATCH(1,C44:N44,0)+1,13))</f>
         <v>12</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
   </sheetData>

</xml_diff>